<commit_message>
chore: remove laudos da raiz e configura o gitignore para relatorios
</commit_message>
<xml_diff>
--- a/Relatorios_Auditoria/Laudo_9_Teste_Quebra_de_Acordo.xlsx
+++ b/Relatorios_Auditoria/Laudo_9_Teste_Quebra_de_Acordo.xlsx
@@ -503,7 +503,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado pelo Nash System v4.0.1 em 02/10/2026 às 22:40</t>
+          <t>Gerado pelo Nash System v4.1.0 em 15/10/2026 às 13:43</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="13" t="n">
-        <v>1.075026788990542</v>
+        <v>1.083842008660264</v>
       </c>
     </row>
     <row r="18">
@@ -659,7 +659,7 @@
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="10" t="n">
-        <v>13760.34289907893</v>
+        <v>13873.17771085138</v>
       </c>
     </row>
     <row r="19">
@@ -673,7 +673,7 @@
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="14" t="n">
-        <v>0.1548999999999997</v>
+        <v>0.1575</v>
       </c>
     </row>
     <row r="20">
@@ -687,7 +687,7 @@
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="10" t="n">
-        <v>2131.477115067323</v>
+        <v>2185.025489459092</v>
       </c>
     </row>
     <row r="21">
@@ -701,7 +701,7 @@
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="12" t="n">
-        <v>15891.82001414625</v>
+        <v>16058.20320031047</v>
       </c>
     </row>
     <row r="23">
@@ -715,7 +715,7 @@
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="10" t="n">
-        <v>1589.182001414626</v>
+        <v>1605.820320031047</v>
       </c>
     </row>
     <row r="24">
@@ -729,7 +729,7 @@
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="10" t="n">
-        <v>3496.200403112176</v>
+        <v>3532.804704068305</v>
       </c>
     </row>
     <row r="25">
@@ -743,7 +743,7 @@
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="10" t="n">
-        <v>2097.720241867306</v>
+        <v>2119.682822440983</v>
       </c>
     </row>
     <row r="26">
@@ -757,7 +757,7 @@
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="10" t="n">
-        <v>2097.720241867306</v>
+        <v>2119.682822440983</v>
       </c>
     </row>
     <row r="27">
@@ -771,7 +771,7 @@
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="12" t="n">
-        <v>25172.64290240766</v>
+        <v>25436.19386929179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>